<commit_message>
integração de card manutenção com base de dados
</commit_message>
<xml_diff>
--- a/backend/dados.xlsx
+++ b/backend/dados.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t xml:space="preserve">status</t>
   </si>
@@ -35,6 +35,18 @@
   </si>
   <si>
     <t xml:space="preserve">taxa_rejeicao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inicio_parada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tempo_parado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">media_paradas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total_paradas</t>
   </si>
   <si>
     <t xml:space="preserve">EM OPERAÇÃO</t>
@@ -47,8 +59,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="hh:mm:ss"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -116,7 +129,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -127,6 +140,14 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -318,7 +339,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.42"/>
@@ -326,6 +347,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13.44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -344,10 +369,22 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>9842</v>
@@ -359,7 +396,19 @@
         <v>740</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.60125</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.00454861111111111</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.00435185185185185</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
integração de cards falhas e produção ao excel
</commit_message>
<xml_diff>
--- a/backend/dados.xlsx
+++ b/backend/dados.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t xml:space="preserve">status</t>
   </si>
@@ -49,19 +49,119 @@
     <t xml:space="preserve">total_paradas</t>
   </si>
   <si>
+    <t xml:space="preserve">status_garrafa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">camera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">confianca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trinca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mancha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sujeira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">risco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">outro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sku</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lote</t>
+  </si>
+  <si>
+    <t xml:space="preserve">envase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">linha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">velocidade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eficiencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">disponibilidade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qualidade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">oee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mtbf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mttr</t>
+  </si>
+  <si>
     <t xml:space="preserve">EM OPERAÇÃO</t>
   </si>
   <si>
     <t xml:space="preserve">7.53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presença de solda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C03: Esquerda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">185 (42,8%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92 (21,1%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">64 (14,7%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">51 (11,8%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31 (7,0%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 (2,9%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMSTEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMSTEL 800ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L240517B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linha 9</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="hh:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yy\ hh:mm"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -129,7 +229,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -142,12 +242,24 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -339,18 +451,32 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:AD2"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="10.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="9.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="10.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="9.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="10.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="10.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="12.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="17.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="11.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="9.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="14.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="0" width="11.05"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -369,22 +495,85 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="0" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>9842</v>
@@ -396,7 +585,7 @@
         <v>740</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.60125</v>
@@ -409,6 +598,69 @@
       </c>
       <c r="I2" s="4" t="n">
         <v>5</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="S2" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="T2" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="U2" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="V2" s="6" t="n">
+        <v>45794.34375</v>
+      </c>
+      <c r="W2" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="X2" s="0" t="n">
+        <v>30000</v>
+      </c>
+      <c r="Y2" s="0" t="n">
+        <v>91.3</v>
+      </c>
+      <c r="Z2" s="0" t="n">
+        <v>86.8</v>
+      </c>
+      <c r="AA2" s="0" t="n">
+        <v>92.6</v>
+      </c>
+      <c r="AB2" s="0" t="n">
+        <v>72.9</v>
+      </c>
+      <c r="AC2" s="7" t="n">
+        <v>0.117210648148148</v>
+      </c>
+      <c r="AD2" s="7" t="n">
+        <v>0.00436342592592593</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajutes de endereço do  mtbf
</commit_message>
<xml_diff>
--- a/backend/dados.xlsx
+++ b/backend/dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aluno.alagoinhas\supervisorio\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B79053A0-54BE-4FF4-BF95-1F064F7297EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E35A29EA-E739-4FF7-97C5-4EB052A1023A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -206,46 +206,46 @@
     <t>51 (11,8%)</t>
   </si>
   <si>
+    <t>12 (2,9%)</t>
+  </si>
+  <si>
+    <t>Linha 9</t>
+  </si>
+  <si>
+    <t>Garrafa trincada</t>
+  </si>
+  <si>
+    <t>Trinca no corpo</t>
+  </si>
+  <si>
+    <t>Garrafa com mancha</t>
+  </si>
+  <si>
+    <t>Soda cáustica</t>
+  </si>
+  <si>
+    <t>Garrafa suja</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Câmera: C03 - Lateral</t>
+  </si>
+  <si>
+    <t>L240517A</t>
+  </si>
+  <si>
+    <t>Confiabildade: 94%</t>
+  </si>
+  <si>
+    <t>AMSTEL</t>
+  </si>
+  <si>
+    <t>AMSTEL 600ml</t>
+  </si>
+  <si>
     <t>31 (7,0%)</t>
-  </si>
-  <si>
-    <t>12 (2,9%)</t>
-  </si>
-  <si>
-    <t>Linha 9</t>
-  </si>
-  <si>
-    <t>Garrafa trincada</t>
-  </si>
-  <si>
-    <t>Trinca no corpo</t>
-  </si>
-  <si>
-    <t>Garrafa com mancha</t>
-  </si>
-  <si>
-    <t>Soda cáustica</t>
-  </si>
-  <si>
-    <t>Garrafa suja</t>
-  </si>
-  <si>
-    <t>OK</t>
-  </si>
-  <si>
-    <t>Câmera: C03 - Lateral</t>
-  </si>
-  <si>
-    <t>SCHIN</t>
-  </si>
-  <si>
-    <t>SCHIN 600ml</t>
-  </si>
-  <si>
-    <t>L240517A</t>
-  </si>
-  <si>
-    <t>Confiabildade: 94%</t>
   </si>
 </sst>
 </file>
@@ -672,10 +672,10 @@
         <v>56</v>
       </c>
       <c r="K2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="L2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="M2" t="s">
         <v>57</v>
@@ -690,40 +690,40 @@
         <v>60</v>
       </c>
       <c r="Q2" t="s">
+        <v>74</v>
+      </c>
+      <c r="R2" t="s">
         <v>61</v>
       </c>
-      <c r="R2" t="s">
-        <v>62</v>
-      </c>
       <c r="S2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="T2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="V2" s="4">
         <v>45794.34375</v>
       </c>
       <c r="W2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="X2">
         <v>24000</v>
       </c>
       <c r="Y2">
-        <v>91.2</v>
+        <v>70</v>
       </c>
       <c r="Z2">
-        <v>86.7</v>
+        <v>81.7</v>
       </c>
       <c r="AA2">
         <v>60</v>
       </c>
       <c r="AB2">
-        <v>72.8</v>
+        <v>63.8</v>
       </c>
       <c r="AC2" s="5">
         <v>0.11686342592592593</v>
@@ -735,10 +735,10 @@
         <v>0.5223726851851852</v>
       </c>
       <c r="AF2" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG2" t="s">
         <v>64</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>65</v>
       </c>
       <c r="AH2">
         <v>6</v>
@@ -750,10 +750,10 @@
         <v>35.4</v>
       </c>
       <c r="AK2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AL2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:38" x14ac:dyDescent="0.25">
@@ -761,10 +761,10 @@
         <v>0.60561342592592593</v>
       </c>
       <c r="AF3" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG3" t="s">
         <v>64</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:38" x14ac:dyDescent="0.25">
@@ -772,10 +772,10 @@
         <v>0.60553240740740744</v>
       </c>
       <c r="AF4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AG4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:38" x14ac:dyDescent="0.25">
@@ -783,10 +783,10 @@
         <v>0.60540509259259256</v>
       </c>
       <c r="AF5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AG5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:38" x14ac:dyDescent="0.25">
@@ -794,10 +794,10 @@
         <v>0.59855324074074079</v>
       </c>
       <c r="AF6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AG6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>